<commit_message>
Clarify RED exclusion counts
</commit_message>
<xml_diff>
--- a/data/processed/seed42_mentor_reply_merged_v5_2026-10-03.xlsx
+++ b/data/processed/seed42_mentor_reply_merged_v5_2026-10-03.xlsx
@@ -2,38 +2,38 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总与结论" sheetId="1" r:id="R6223e0d3ebed4b92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact核查30条" sheetId="2" r:id="R65bb50727ffe4942"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReferenceErrorDetection核查30条" sheetId="3" r:id="R3beea912e2564eec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云复核说明" sheetId="4" r:id="R58606cc32ae5448f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云确认说明" sheetId="5" r:id="R02d6f02452d74b30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补定位说明" sheetId="6" r:id="R54fb8ed60a5e42ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED补证与排除说明" sheetId="7" r:id="Rccb7f16ed3624a04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED30补定位说明" sheetId="8" r:id="R070b74840d07452a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED8补定位说明" sheetId="9" r:id="R7102e5ead69b489b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED4补定位说明" sheetId="10" r:id="R08d3c29c5aa24c6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED10补定位与排除说明" sheetId="11" r:id="Rb68d6e8e252a466b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact补证说明_2026-10-02" sheetId="12" r:id="R97d216903a244b37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED11补定位说明" sheetId="13" r:id="Rcfdecc737aca4898"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED20补定位说明" sheetId="14" r:id="Rcaac1e5a5672415b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED12补定位说明" sheetId="15" r:id="R6254183fe76449ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED7补定位说明" sheetId="16" r:id="R86670bc28d9848b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED14补定位说明" sheetId="17" r:id="R84ae782e947c41f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED3补定位说明" sheetId="18" r:id="R3c0fbc98c7f34000"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED18补定位说明" sheetId="19" r:id="R6238442bb83a49b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED5补定位说明" sheetId="20" r:id="R925020ebecca4112"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED9补定位说明" sheetId="21" r:id="R8d7f7cbc75264fdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED13补定位说明" sheetId="22" r:id="Re9668080449e4134"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED28补定位说明" sheetId="23" r:id="Rc57f793e53dc4ef7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED剩余补定位说明" sheetId="24" r:id="R4d4e2d4009ea4a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact两条补证说明" sheetId="25" r:id="Rdb0621cbcd4f403d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规范化预合并说明" sheetId="26" r:id="Rb701504fe6a3478b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄裁决记录_2026-10-03" sheetId="27" r:id="R9945ff48848a4f99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="许可更正说明_2026-10-03" sheetId="28" r:id="R68caa6e69d24408f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补证记录_2026-10-03" sheetId="29" r:id="R9c23d6aba8274b39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前快照说明_2026-10-03" sheetId="30" r:id="Re4eb84e2ff3b4af2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄回传核对_2026-10-03" sheetId="31" r:id="R1db5be757f5f40bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待裁决分歧_2026-10-03" sheetId="32" r:id="R2fb1dc136b014f5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总与结论" sheetId="1" r:id="Ra132f498f1214f13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact核查30条" sheetId="2" r:id="Re6a4848f66344b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReferenceErrorDetection核查30条" sheetId="3" r:id="R138c2f64c0554401"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云复核说明" sheetId="4" r:id="R9c2d0a0caf0145b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云确认说明" sheetId="5" r:id="R924d48e05a8e4078"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补定位说明" sheetId="6" r:id="R30f8192359774104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED补证与排除说明" sheetId="7" r:id="R9427c5fe878d4894"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED30补定位说明" sheetId="8" r:id="Rd1d5d15d06ab4186"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED8补定位说明" sheetId="9" r:id="R4c11f82cbc1b4667"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED4补定位说明" sheetId="10" r:id="Re6c5016f463d416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED10补定位与排除说明" sheetId="11" r:id="R57fd2db4593a4d06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact补证说明_2026-10-02" sheetId="12" r:id="R9619fe8d59284f7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED11补定位说明" sheetId="13" r:id="Rd484336fee64452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED20补定位说明" sheetId="14" r:id="Rcd91b2f38a9e4012"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED12补定位说明" sheetId="15" r:id="R9f6761fde7be431d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED7补定位说明" sheetId="16" r:id="R38257a225eee44fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED14补定位说明" sheetId="17" r:id="R8390b8e3a66a415b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED3补定位说明" sheetId="18" r:id="Ra9141731ac6e4754"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED18补定位说明" sheetId="19" r:id="R869322bf74f34bf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED5补定位说明" sheetId="20" r:id="Reb53c14a29364d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED9补定位说明" sheetId="21" r:id="Rfd770ead70044dd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED13补定位说明" sheetId="22" r:id="Raa966200c6434578"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED28补定位说明" sheetId="23" r:id="R2b182bc125224e48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED剩余补定位说明" sheetId="24" r:id="R69f5f34122314d84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact两条补证说明" sheetId="25" r:id="R39eb47b9517d467e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规范化预合并说明" sheetId="26" r:id="R8642d8e5719c4efa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄裁决记录_2026-10-03" sheetId="27" r:id="Rc26939ec02804343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="许可更正说明_2026-10-03" sheetId="28" r:id="Rdcfe03e6e5534b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补证记录_2026-10-03" sheetId="29" r:id="Rb9ce140c8b2741d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前快照说明_2026-10-03" sheetId="30" r:id="R7f13bd5d91484393"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄回传核对_2026-10-03" sheetId="31" r:id="R29736d1ae1074736"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待裁决分歧_2026-10-03" sheetId="32" r:id="R88a1e2971354458b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11666,7 +11666,7 @@
         <x:v>RED 双方标签</x:v>
       </x:c>
       <x:c r="B7" s="101" t="str">
-        <x:v>25 条一致，3 条不一致；RED:2、RED:6 仍为不可用/排除</x:v>
+        <x:v>28 条有双方三分类标签：25 条一致，3 条不一致；RED:2、RED:6、RED:10、RED:21 均为不可用/排除，因此 26 条正式可用记录中为 23 条一致、3 条不一致</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">

</xml_diff>

<commit_message>
Refresh merged workbook summary
</commit_message>
<xml_diff>
--- a/data/processed/seed42_mentor_reply_merged_v5_2026-10-03.xlsx
+++ b/data/processed/seed42_mentor_reply_merged_v5_2026-10-03.xlsx
@@ -2,38 +2,38 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总与结论" sheetId="1" r:id="Ra132f498f1214f13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact核查30条" sheetId="2" r:id="Re6a4848f66344b14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReferenceErrorDetection核查30条" sheetId="3" r:id="R138c2f64c0554401"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云复核说明" sheetId="4" r:id="R9c2d0a0caf0145b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云确认说明" sheetId="5" r:id="R924d48e05a8e4078"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补定位说明" sheetId="6" r:id="R30f8192359774104"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED补证与排除说明" sheetId="7" r:id="R9427c5fe878d4894"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED30补定位说明" sheetId="8" r:id="Rd1d5d15d06ab4186"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED8补定位说明" sheetId="9" r:id="R4c11f82cbc1b4667"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED4补定位说明" sheetId="10" r:id="Re6c5016f463d416a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED10补定位与排除说明" sheetId="11" r:id="R57fd2db4593a4d06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact补证说明_2026-10-02" sheetId="12" r:id="R9619fe8d59284f7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED11补定位说明" sheetId="13" r:id="Rd484336fee64452f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED20补定位说明" sheetId="14" r:id="Rcd91b2f38a9e4012"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED12补定位说明" sheetId="15" r:id="R9f6761fde7be431d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED7补定位说明" sheetId="16" r:id="R38257a225eee44fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED14补定位说明" sheetId="17" r:id="R8390b8e3a66a415b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED3补定位说明" sheetId="18" r:id="Ra9141731ac6e4754"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED18补定位说明" sheetId="19" r:id="R869322bf74f34bf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED5补定位说明" sheetId="20" r:id="Reb53c14a29364d70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED9补定位说明" sheetId="21" r:id="Rfd770ead70044dd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED13补定位说明" sheetId="22" r:id="Raa966200c6434578"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED28补定位说明" sheetId="23" r:id="R2b182bc125224e48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED剩余补定位说明" sheetId="24" r:id="R69f5f34122314d84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact两条补证说明" sheetId="25" r:id="R39eb47b9517d467e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规范化预合并说明" sheetId="26" r:id="R8642d8e5719c4efa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄裁决记录_2026-10-03" sheetId="27" r:id="Rc26939ec02804343"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="许可更正说明_2026-10-03" sheetId="28" r:id="Rdcfe03e6e5534b46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补证记录_2026-10-03" sheetId="29" r:id="Rb9ce140c8b2741d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前快照说明_2026-10-03" sheetId="30" r:id="R7f13bd5d91484393"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄回传核对_2026-10-03" sheetId="31" r:id="R29736d1ae1074736"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待裁决分歧_2026-10-03" sheetId="32" r:id="R88a1e2971354458b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总与结论" sheetId="1" r:id="R980cf90227c54ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact核查30条" sheetId="2" r:id="R2c15125fd0174985"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReferenceErrorDetection核查30条" sheetId="3" r:id="R539058fefd2746af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云复核说明" sheetId="4" r:id="Raba7cf1e62b443ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云确认说明" sheetId="5" r:id="R9d0c53bd63694121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补定位说明" sheetId="6" r:id="Rd50f79c8b75748ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED补证与排除说明" sheetId="7" r:id="Rc236a86d91c14174"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED30补定位说明" sheetId="8" r:id="R92cf9bf7501748b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED8补定位说明" sheetId="9" r:id="Rf5817994115546c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED4补定位说明" sheetId="10" r:id="R2ceeb1266a3a4595"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED10补定位与排除说明" sheetId="11" r:id="R76ec1c67cc3241fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact补证说明_2026-10-02" sheetId="12" r:id="Rb4b36e0fd6a94859"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED11补定位说明" sheetId="13" r:id="Rb78e14a358014cd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED20补定位说明" sheetId="14" r:id="Rdd6d86178d0440c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED12补定位说明" sheetId="15" r:id="R03d032519cba4aa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED7补定位说明" sheetId="16" r:id="Rab220e7ecc7a493e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED14补定位说明" sheetId="17" r:id="Rb1ad28ef6a8842ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED3补定位说明" sheetId="18" r:id="R673b5b8d5ee54742"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED18补定位说明" sheetId="19" r:id="Ra77b9907e5ed4b0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED5补定位说明" sheetId="20" r:id="Re098840d428e46d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED9补定位说明" sheetId="21" r:id="R27b24e18aed94d21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED13补定位说明" sheetId="22" r:id="R381f04292a9843ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED28补定位说明" sheetId="23" r:id="Raa57027be1d04561"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED剩余补定位说明" sheetId="24" r:id="Rdf096f14467f431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact两条补证说明" sheetId="25" r:id="R6c75d11438614693"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规范化预合并说明" sheetId="26" r:id="Rb8f2f4e5f4384f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄裁决记录_2026-10-03" sheetId="27" r:id="R1214c0a79bb04af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="许可更正说明_2026-10-03" sheetId="28" r:id="R41299d06dd194276"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补证记录_2026-10-03" sheetId="29" r:id="R82f03812a4e04670"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前快照说明_2026-10-03" sheetId="30" r:id="Rc9c82ee849894520"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄回传核对_2026-10-03" sheetId="31" r:id="R2c270aefe14b4acc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待裁决分歧_2026-10-03" sheetId="32" r:id="Rc0b8ea0b9bb54409"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -854,7 +854,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="str">
-        <x:v>  30条抽样：17条双方标签与裁决已完成（ACCURATE10/NOT_ACCURATE7）；13条仍待陈明进确认</x:v>
+        <x:v>  30条抽样：双方独立标签已全部回收；24条一致、6条分歧；其中17条已有裁决，13条待裁决。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>

<commit_message>
Clarify adjudication and consensus status
</commit_message>
<xml_diff>
--- a/data/processed/seed42_mentor_reply_merged_v5_2026-10-03.xlsx
+++ b/data/processed/seed42_mentor_reply_merged_v5_2026-10-03.xlsx
@@ -2,38 +2,39 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总与结论" sheetId="1" r:id="R980cf90227c54ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact核查30条" sheetId="2" r:id="R2c15125fd0174985"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReferenceErrorDetection核查30条" sheetId="3" r:id="R539058fefd2746af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云复核说明" sheetId="4" r:id="Raba7cf1e62b443ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云确认说明" sheetId="5" r:id="R9d0c53bd63694121"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补定位说明" sheetId="6" r:id="Rd50f79c8b75748ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED补证与排除说明" sheetId="7" r:id="Rc236a86d91c14174"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED30补定位说明" sheetId="8" r:id="R92cf9bf7501748b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED8补定位说明" sheetId="9" r:id="Rf5817994115546c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED4补定位说明" sheetId="10" r:id="R2ceeb1266a3a4595"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED10补定位与排除说明" sheetId="11" r:id="R76ec1c67cc3241fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact补证说明_2026-10-02" sheetId="12" r:id="Rb4b36e0fd6a94859"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED11补定位说明" sheetId="13" r:id="Rb78e14a358014cd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED20补定位说明" sheetId="14" r:id="Rdd6d86178d0440c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED12补定位说明" sheetId="15" r:id="R03d032519cba4aa4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED7补定位说明" sheetId="16" r:id="Rab220e7ecc7a493e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED14补定位说明" sheetId="17" r:id="Rb1ad28ef6a8842ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED3补定位说明" sheetId="18" r:id="R673b5b8d5ee54742"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED18补定位说明" sheetId="19" r:id="Ra77b9907e5ed4b0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED5补定位说明" sheetId="20" r:id="Re098840d428e46d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED9补定位说明" sheetId="21" r:id="R27b24e18aed94d21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED13补定位说明" sheetId="22" r:id="R381f04292a9843ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED28补定位说明" sheetId="23" r:id="Raa57027be1d04561"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED剩余补定位说明" sheetId="24" r:id="Rdf096f14467f431a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact两条补证说明" sheetId="25" r:id="R6c75d11438614693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规范化预合并说明" sheetId="26" r:id="Rb8f2f4e5f4384f22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄裁决记录_2026-10-03" sheetId="27" r:id="R1214c0a79bb04af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="许可更正说明_2026-10-03" sheetId="28" r:id="R41299d06dd194276"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补证记录_2026-10-03" sheetId="29" r:id="R82f03812a4e04670"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前快照说明_2026-10-03" sheetId="30" r:id="Rc9c82ee849894520"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄回传核对_2026-10-03" sheetId="31" r:id="R2c270aefe14b4acc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待裁决分歧_2026-10-03" sheetId="32" r:id="Rc0b8ea0b9bb54409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总与结论" sheetId="1" r:id="Rfc3ff26222bd44cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact核查30条" sheetId="2" r:id="Rdce1e8197c024b34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReferenceErrorDetection核查30条" sheetId="3" r:id="R472adef2d82d4192"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云复核说明" sheetId="4" r:id="Rcd37ec9ba7744588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="李云确认说明" sheetId="5" r:id="R40c97efcdb384fcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补定位说明" sheetId="6" r:id="Rbae55747bccf45a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED补证与排除说明" sheetId="7" r:id="R9a53a31f645e4ce3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED30补定位说明" sheetId="8" r:id="Ra582e96a3ad14512"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED8补定位说明" sheetId="9" r:id="R35c7bf51addb4cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED4补定位说明" sheetId="10" r:id="Ra7e8dc153d0b44e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED10补定位与排除说明" sheetId="11" r:id="Rb5dd5af975b547db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact补证说明_2026-10-02" sheetId="12" r:id="R2444aceca4b249b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED11补定位说明" sheetId="13" r:id="R8fafa267d3c34031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED20补定位说明" sheetId="14" r:id="R21a8dcd8afc24fa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED12补定位说明" sheetId="15" r:id="R22c37d6f97b8476c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED7补定位说明" sheetId="16" r:id="R5b1eedad59e74b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED14补定位说明" sheetId="17" r:id="R1be92e239c1c4b6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED3补定位说明" sheetId="18" r:id="R6e2653c083ee48a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED18补定位说明" sheetId="19" r:id="R833f9c91aad84601"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED5补定位说明" sheetId="20" r:id="R43250576f8c742ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED9补定位说明" sheetId="21" r:id="R7e325c5ac392468a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED13补定位说明" sheetId="22" r:id="R235bd18d7db14895"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED28补定位说明" sheetId="23" r:id="Ree0183d4fa0045f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED剩余补定位说明" sheetId="24" r:id="R6d31ab5442b84189"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SciFact两条补证说明" sheetId="25" r:id="Ree143b739eba444e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规范化预合并说明" sheetId="26" r:id="Re132724dd79b45ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄裁决记录_2026-10-03" sheetId="27" r:id="Rfbfdb907e3c347d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="许可更正说明_2026-10-03" sheetId="28" r:id="R2bc8fd93882c4501"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED全文补证记录_2026-10-03" sheetId="29" r:id="Rd9f5c647d9c04220"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前快照说明_2026-10-03" sheetId="30" r:id="R4bc1ba9019eb4ab9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="师兄回传核对_2026-10-03" sheetId="31" r:id="R1022ebe8cde84649"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待裁决分歧_2026-10-03" sheetId="32" r:id="Rd69be80675e04001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="一致但待登记_2026-10-03" sheetId="33" r:id="Rad56a46ef818470c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,7 +87,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="31">
+  <x:fills count="32">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -238,6 +239,11 @@
         <x:fgColor rgb="FFC65911"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF548235"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -273,7 +279,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="127">
+  <x:cellXfs count="131">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0"/>
@@ -523,6 +529,14 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -11698,7 +11712,9 @@
     <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -11715,6 +11731,12 @@
         <x:v>annotator_2_label</x:v>
       </x:c>
       <x:c r="E1" s="126" t="str">
+        <x:v>project_label</x:v>
+      </x:c>
+      <x:c r="F1" s="126" t="str">
+        <x:v>adjudicated_label</x:v>
+      </x:c>
+      <x:c r="G1" s="126" t="str">
         <x:v>状态</x:v>
       </x:c>
     </x:row>
@@ -11732,7 +11754,13 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="E2" s="101" t="str">
-        <x:v>待裁决</x:v>
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="F2" s="101" t="str">
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="G2" s="101" t="str">
+        <x:v>已有裁决（继承 v4）</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
@@ -11749,7 +11777,13 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="E3" s="101" t="str">
-        <x:v>待裁决</x:v>
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="F3" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="G3" s="101" t="str">
+        <x:v>已有裁决（继承 v4）</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
@@ -11766,7 +11800,13 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="E4" s="101" t="str">
-        <x:v>待裁决</x:v>
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="F4" s="101" t="str">
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="G4" s="101" t="str">
+        <x:v>已有裁决（继承 v4）</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
@@ -11783,7 +11823,13 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="E5" s="101" t="str">
-        <x:v>待裁决</x:v>
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="F5" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="G5" s="101" t="str">
+        <x:v>已有裁决（继承 v4）</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
@@ -11800,7 +11846,13 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="E6" s="101" t="str">
-        <x:v>待裁决</x:v>
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="F6" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="G6" s="101" t="str">
+        <x:v>已有裁决（继承 v4）</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -11817,7 +11869,13 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="E7" s="101" t="str">
-        <x:v>待裁决</x:v>
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="F7" s="101" t="str">
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="G7" s="101" t="str">
+        <x:v>已有裁决（继承 v4）</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -11834,7 +11892,13 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="E8" s="101" t="str">
-        <x:v>待裁决</x:v>
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="F8" s="101" t="str">
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="G8" s="101" t="str">
+        <x:v>已有裁决（继承 v4）</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -11851,7 +11915,13 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="E9" s="101" t="str">
-        <x:v>待裁决</x:v>
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="F9" s="101" t="str">
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="G9" s="101" t="str">
+        <x:v>已有裁决（继承 v4）</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
@@ -11868,7 +11938,301 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="E10" s="101" t="str">
-        <x:v>待裁决</x:v>
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="F10" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="G10" s="101" t="str">
+        <x:v>已有裁决（继承 v4）</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="130" t="str">
+        <x:v>数据集</x:v>
+      </x:c>
+      <x:c r="B1" s="130" t="str">
+        <x:v>citation_id</x:v>
+      </x:c>
+      <x:c r="C1" s="130" t="str">
+        <x:v>双方标签</x:v>
+      </x:c>
+      <x:c r="D1" s="130" t="str">
+        <x:v>证据状态</x:v>
+      </x:c>
+      <x:c r="E1" s="130" t="str">
+        <x:v>当前项目标签</x:v>
+      </x:c>
+      <x:c r="F1" s="130" t="str">
+        <x:v>当前裁决标签</x:v>
+      </x:c>
+      <x:c r="G1" s="130" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B2" s="101" t="str">
+        <x:v>SciFact:train-389</x:v>
+      </x:c>
+      <x:c r="C2" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="D2" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E2" s="101" t="str"/>
+      <x:c r="F2" s="101" t="str"/>
+      <x:c r="G2" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="30" customHeight="1">
+      <x:c r="A3" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B3" s="101" t="str">
+        <x:v>SciFact:train-876</x:v>
+      </x:c>
+      <x:c r="C3" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="D3" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E3" s="101" t="str"/>
+      <x:c r="F3" s="101" t="str"/>
+      <x:c r="G3" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B4" s="101" t="str">
+        <x:v>SciFact:train-486</x:v>
+      </x:c>
+      <x:c r="C4" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="D4" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E4" s="101" t="str"/>
+      <x:c r="F4" s="101" t="str"/>
+      <x:c r="G4" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B5" s="101" t="str">
+        <x:v>SciFact:train-361</x:v>
+      </x:c>
+      <x:c r="C5" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="D5" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E5" s="101" t="str"/>
+      <x:c r="F5" s="101" t="str"/>
+      <x:c r="G5" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="A6" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B6" s="101" t="str">
+        <x:v>SciFact:dev-238</x:v>
+      </x:c>
+      <x:c r="C6" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="D6" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E6" s="101" t="str"/>
+      <x:c r="F6" s="101" t="str"/>
+      <x:c r="G6" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B7" s="101" t="str">
+        <x:v>SciFact:train-96</x:v>
+      </x:c>
+      <x:c r="C7" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="D7" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E7" s="101" t="str"/>
+      <x:c r="F7" s="101" t="str"/>
+      <x:c r="G7" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B8" s="101" t="str">
+        <x:v>SciFact:train-91</x:v>
+      </x:c>
+      <x:c r="C8" s="101" t="str">
+        <x:v>IRRELEVANT</x:v>
+      </x:c>
+      <x:c r="D8" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E8" s="101" t="str"/>
+      <x:c r="F8" s="101" t="str"/>
+      <x:c r="G8" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B9" s="101" t="str">
+        <x:v>SciFact:train-817</x:v>
+      </x:c>
+      <x:c r="C9" s="101" t="str">
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="D9" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E9" s="101" t="str"/>
+      <x:c r="F9" s="101" t="str"/>
+      <x:c r="G9" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B10" s="101" t="str">
+        <x:v>SciFact:train-81</x:v>
+      </x:c>
+      <x:c r="C10" s="101" t="str">
+        <x:v>IRRELEVANT</x:v>
+      </x:c>
+      <x:c r="D10" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E10" s="101" t="str"/>
+      <x:c r="F10" s="101" t="str"/>
+      <x:c r="G10" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B11" s="101" t="str">
+        <x:v>SciFact:train-777</x:v>
+      </x:c>
+      <x:c r="C11" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="D11" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E11" s="101" t="str"/>
+      <x:c r="F11" s="101" t="str"/>
+      <x:c r="G11" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B12" s="101" t="str">
+        <x:v>SciFact:train-20</x:v>
+      </x:c>
+      <x:c r="C12" s="101" t="str">
+        <x:v>NOT_ACCURATE</x:v>
+      </x:c>
+      <x:c r="D12" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E12" s="101" t="str"/>
+      <x:c r="F12" s="101" t="str"/>
+      <x:c r="G12" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B13" s="101" t="str">
+        <x:v>SciFact:train-1212</x:v>
+      </x:c>
+      <x:c r="C13" s="101" t="str">
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="D13" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E13" s="101" t="str"/>
+      <x:c r="F13" s="101" t="str"/>
+      <x:c r="G13" s="101" t="str">
+        <x:v>待登记共识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="101" t="str">
+        <x:v>SciFact</x:v>
+      </x:c>
+      <x:c r="B14" s="101" t="str">
+        <x:v>SciFact:train-1195</x:v>
+      </x:c>
+      <x:c r="C14" s="101" t="str">
+        <x:v>ACCURATE</x:v>
+      </x:c>
+      <x:c r="D14" s="101" t="str">
+        <x:v>已定位</x:v>
+      </x:c>
+      <x:c r="E14" s="101" t="str"/>
+      <x:c r="F14" s="101" t="str"/>
+      <x:c r="G14" s="101" t="str">
+        <x:v>待登记共识</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>